<commit_message>
Align active map scoring with available GeoJSON files and penalize extra features
</commit_message>
<xml_diff>
--- a/map_similarity_results.xlsx
+++ b/map_similarity_results.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>matched exact (name + geometry type) / Reference Features</t>
+          <t>matched exact (name + geometry type) / (Reference Features + Extra Features)</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -709,31 +709,31 @@
         <v>1</v>
       </c>
       <c r="O3" t="n">
-        <v>1</v>
+        <v>0.839</v>
       </c>
       <c r="P3" t="n">
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>1</v>
+        <v>0.833</v>
       </c>
       <c r="R3" t="n">
-        <v>1</v>
+        <v>0.738</v>
       </c>
       <c r="S3" t="n">
-        <v>1</v>
+        <v>0.86</v>
       </c>
       <c r="T3" t="n">
-        <v>1</v>
+        <v>0.733</v>
       </c>
       <c r="U3" t="n">
-        <v>1</v>
+        <v>0.907</v>
       </c>
       <c r="V3" t="n">
-        <v>1</v>
+        <v>0.864</v>
       </c>
       <c r="W3" t="n">
-        <v>100</v>
+        <v>86.38</v>
       </c>
     </row>
     <row r="4">
@@ -764,7 +764,7 @@
         <v>6</v>
       </c>
       <c r="G4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H4" t="n">
         <v>6</v>
@@ -773,11 +773,11 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>All baseline features were matched; no extra participant features remained.</t>
+          <t>0 baseline features were unmatched and 1 participant features were unmatched. Missing sample: n/a. Extra sample: n/a.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -791,34 +791,34 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>1</v>
+        <v>0.857</v>
       </c>
       <c r="O4" t="n">
-        <v>1</v>
+        <v>0.972</v>
       </c>
       <c r="P4" t="n">
-        <v>1</v>
+        <v>0.984</v>
       </c>
       <c r="Q4" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="R4" t="n">
-        <v>1</v>
+        <v>0.946</v>
       </c>
       <c r="S4" t="n">
-        <v>1</v>
+        <v>0.969</v>
       </c>
       <c r="T4" t="n">
-        <v>1</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="U4" t="n">
-        <v>1</v>
+        <v>0.983</v>
       </c>
       <c r="V4" t="n">
-        <v>1</v>
+        <v>0.954</v>
       </c>
       <c r="W4" t="n">
-        <v>100</v>
+        <v>95.43000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -879,7 +879,7 @@
         <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>0.882</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
@@ -888,22 +888,22 @@
         <v>1</v>
       </c>
       <c r="R5" t="n">
-        <v>1</v>
+        <v>0.831</v>
       </c>
       <c r="S5" t="n">
-        <v>1</v>
+        <v>0.761</v>
       </c>
       <c r="T5" t="n">
-        <v>1</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="U5" t="n">
-        <v>1</v>
+        <v>0.882</v>
       </c>
       <c r="V5" t="n">
-        <v>1</v>
+        <v>0.911</v>
       </c>
       <c r="W5" t="n">
-        <v>100</v>
+        <v>91.11</v>
       </c>
     </row>
     <row r="6">
@@ -934,20 +934,20 @@
         <v>6</v>
       </c>
       <c r="G6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>All baseline features were matched; no extra participant features remained.</t>
+          <t>1 baseline features were unmatched and 0 participant features were unmatched. Missing sample: Storage Room. Extra sample: n/a.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -961,34 +961,34 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>1</v>
+        <v>0.833</v>
       </c>
       <c r="O6" t="n">
-        <v>1</v>
+        <v>0.825</v>
       </c>
       <c r="P6" t="n">
-        <v>1</v>
+        <v>0.92</v>
       </c>
       <c r="Q6" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="R6" t="n">
-        <v>1</v>
+        <v>0.703</v>
       </c>
       <c r="S6" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="T6" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="U6" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="V6" t="n">
-        <v>1</v>
+        <v>0.825</v>
       </c>
       <c r="W6" t="n">
-        <v>100</v>
+        <v>82.47</v>
       </c>
     </row>
     <row r="7">
@@ -1134,31 +1134,31 @@
         <v>1</v>
       </c>
       <c r="O8" t="n">
-        <v>1</v>
+        <v>0.986</v>
       </c>
       <c r="P8" t="n">
-        <v>1</v>
+        <v>0.973</v>
       </c>
       <c r="Q8" t="n">
         <v>1</v>
       </c>
       <c r="R8" t="n">
-        <v>1</v>
+        <v>0.988</v>
       </c>
       <c r="S8" t="n">
-        <v>1</v>
+        <v>0.991</v>
       </c>
       <c r="T8" t="n">
         <v>1</v>
       </c>
       <c r="U8" t="n">
-        <v>1</v>
+        <v>0.995</v>
       </c>
       <c r="V8" t="n">
-        <v>1</v>
+        <v>0.992</v>
       </c>
       <c r="W8" t="n">
-        <v>100</v>
+        <v>99.16</v>
       </c>
     </row>
   </sheetData>
@@ -1172,7 +1172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W16"/>
+  <dimension ref="A1:W15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>matched exact (name + geometry type) / Reference Features</t>
+          <t>matched exact (name + geometry type) / (Reference Features + Extra Features)</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1522,20 +1522,20 @@
         <v>6</v>
       </c>
       <c r="G4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>All baseline features were matched; no extra participant features remained.</t>
+          <t>1 baseline features were unmatched and 0 participant features were unmatched. Missing sample: Front Desk. Extra sample: n/a.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1549,7 +1549,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>1</v>
+        <v>0.833</v>
       </c>
       <c r="O4" t="n">
         <v>1</v>
@@ -1573,10 +1573,10 @@
         <v>1</v>
       </c>
       <c r="V4" t="n">
-        <v>1</v>
+        <v>0.979</v>
       </c>
       <c r="W4" t="n">
-        <v>100</v>
+        <v>97.91</v>
       </c>
     </row>
     <row r="5">
@@ -1591,16 +1591,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2, 3</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>p7/Sighted_p7_Spatial_Knowledge_map_2.geojson</t>
+          <t>p7/Sighted_p7_Spatial_Knowledge_map_3.geojson</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Map 2</t>
+          <t>Map 3</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1637,7 +1637,7 @@
         <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>0.979</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
@@ -1646,22 +1646,22 @@
         <v>1</v>
       </c>
       <c r="R5" t="n">
-        <v>1</v>
+        <v>0.92</v>
       </c>
       <c r="S5" t="n">
-        <v>1</v>
+        <v>0.973</v>
       </c>
       <c r="T5" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="U5" t="n">
-        <v>1</v>
+        <v>0.979</v>
       </c>
       <c r="V5" t="n">
-        <v>1</v>
+        <v>0.956</v>
       </c>
       <c r="W5" t="n">
-        <v>100</v>
+        <v>95.64</v>
       </c>
     </row>
     <row r="6">
@@ -1672,11 +1672,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>p7</t>
+          <t>p8</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>p7/Sighted_p7_Spatial_Knowledge_map_3.geojson</t>
+          <t>p8/Sighted_p8_Spatial_Knowledge_map_2.geojson</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Map 3</t>
+          <t>Map 2</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2, 3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1947,7 +1947,7 @@
         <v>6</v>
       </c>
       <c r="G9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H9" t="n">
         <v>6</v>
@@ -1956,11 +1956,11 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>All baseline features were matched; no extra participant features remained.</t>
+          <t>0 baseline features were unmatched and 1 participant features were unmatched. Missing sample: n/a. Extra sample: n/a.</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1974,7 +1974,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>0.857</v>
       </c>
       <c r="O9" t="n">
         <v>1</v>
@@ -1998,10 +1998,10 @@
         <v>1</v>
       </c>
       <c r="V9" t="n">
-        <v>1</v>
+        <v>0.982</v>
       </c>
       <c r="W9" t="n">
-        <v>100</v>
+        <v>98.20999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -2117,7 +2117,7 @@
         <v>6</v>
       </c>
       <c r="G11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H11" t="n">
         <v>6</v>
@@ -2126,11 +2126,11 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>All baseline features were matched; no extra participant features remained.</t>
+          <t>0 baseline features were unmatched and 1 participant features were unmatched. Missing sample: n/a. Extra sample: n/a.</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -2144,7 +2144,7 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>1</v>
+        <v>0.857</v>
       </c>
       <c r="O11" t="n">
         <v>1</v>
@@ -2168,10 +2168,10 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>1</v>
+        <v>0.982</v>
       </c>
       <c r="W11" t="n">
-        <v>100</v>
+        <v>98.20999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2, 3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -2287,7 +2287,7 @@
         <v>6</v>
       </c>
       <c r="G13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H13" t="n">
         <v>6</v>
@@ -2296,11 +2296,11 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>All baseline features were matched; no extra participant features remained.</t>
+          <t>0 baseline features were unmatched and 1 participant features were unmatched. Missing sample: n/a. Extra sample: n/a.</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>1</v>
+        <v>0.857</v>
       </c>
       <c r="O13" t="n">
         <v>1</v>
@@ -2338,10 +2338,10 @@
         <v>1</v>
       </c>
       <c r="V13" t="n">
-        <v>1</v>
+        <v>0.982</v>
       </c>
       <c r="W13" t="n">
-        <v>100</v>
+        <v>98.20999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -2352,11 +2352,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>p12</t>
+          <t>p13</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -2365,14 +2365,14 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>p12/Sighted_p12_Spatial_Knowledge_map_3.geojson</t>
+          <t>p13/Sighted_p13_Spatial_Knowledge_map_2.geojson</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>6</v>
       </c>
       <c r="G14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H14" t="n">
         <v>6</v>
@@ -2381,16 +2381,16 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>All baseline features were matched; no extra participant features remained.</t>
+          <t>0 baseline features were unmatched and 1 participant features were unmatched. Missing sample: n/a. Extra sample: n/a.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Map 3</t>
+          <t>Map 2</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2399,7 +2399,7 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>0.857</v>
       </c>
       <c r="O14" t="n">
         <v>1</v>
@@ -2423,10 +2423,10 @@
         <v>1</v>
       </c>
       <c r="V14" t="n">
-        <v>1</v>
+        <v>0.982</v>
       </c>
       <c r="W14" t="n">
-        <v>100</v>
+        <v>98.20999999999999</v>
       </c>
     </row>
     <row r="15">
@@ -2441,7 +2441,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>p13/Sighted_p13_Spatial_Knowledge_map_2.geojson</t>
+          <t>p13/Sighted_p13_Spatial_Knowledge_map_3.geojson</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Map 2</t>
+          <t>Map 3</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2511,91 +2511,6 @@
         <v>1</v>
       </c>
       <c r="W15" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>sighted</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>p13</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>2, 3</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>p13/Sighted_p13_Spatial_Knowledge_map_3.geojson</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>6</v>
-      </c>
-      <c r="G16" t="n">
-        <v>6</v>
-      </c>
-      <c r="H16" t="n">
-        <v>6</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>All baseline features were matched; no extra participant features remained.</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Map 3</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Feature names match expected map signature.</t>
-        </is>
-      </c>
-      <c r="N16" t="n">
-        <v>1</v>
-      </c>
-      <c r="O16" t="n">
-        <v>1</v>
-      </c>
-      <c r="P16" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>1</v>
-      </c>
-      <c r="R16" t="n">
-        <v>1</v>
-      </c>
-      <c r="S16" t="n">
-        <v>1</v>
-      </c>
-      <c r="T16" t="n">
-        <v>1</v>
-      </c>
-      <c r="U16" t="n">
-        <v>1</v>
-      </c>
-      <c r="V16" t="n">
-        <v>1</v>
-      </c>
-      <c r="W16" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>